<commit_message>
Add distribution/podcast checklist and wire 3-9 into calendar, KPI sheet and dashboard
- templates/music_distribution_podcast_checklist.md: go/no-go on audio
  sources, distributor choice, first-album metadata sheet, Official
  Artist Channel steps, podcast hosting, RSS submission and verification
- Calendar: one distribution task per week (4 new rows, 32 total)
- KPI sheet: YouTube Music and podcast traffic-share rows
- Dashboard: new finding when traffic sources lack YouTube Music/podcast
- Plan 3-9 and README link to the new checklist

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C2dffSHYa7wwyhksGy8dMJ
</commit_message>
<xml_diff>
--- a/calendar/4week_calendar.xlsx
+++ b/calendar/4week_calendar.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -882,27 +882,27 @@
         </is>
       </c>
       <c r="C11" s="8">
-        <f>$B$2+6</f>
+        <f>$B$2+5</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>기준선 기록: 노출·CTR·AVD·트래픽 소스</t>
+          <t>음원 출처 정리(자체 제작·독점만), 유통사·팟캐스트 호스팅 계정 개설</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W0</t>
+          <t>출처표, 계정</t>
         </is>
       </c>
       <c r="H11" s="9" t="n"/>
@@ -912,36 +912,36 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>신규 콘텐츠 + A/B</t>
+          <t>점검·세팅</t>
         </is>
       </c>
       <c r="C12" s="8">
-        <f>$B$2+7</f>
+        <f>$B$2+6</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>설문 결과 발표 + 화요일 공개 예고</t>
+          <t>기준선 기록: 노출·CTR·AVD·트래픽 소스</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>게시글</t>
+          <t>KPI 시트 W0</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
@@ -960,27 +960,27 @@
         </is>
       </c>
       <c r="C13" s="8">
-        <f>$B$2+8</f>
+        <f>$B$2+7</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #1 공개 (새 제목 공식, 썸네일 A/B 3종)</t>
+          <t>설문 결과 발표 + 화요일 공개 예고</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>CTR 48h</t>
+          <t>게시글</t>
         </is>
       </c>
       <c r="H13" s="9" t="n"/>
@@ -999,27 +999,27 @@
         </is>
       </c>
       <c r="C14" s="8">
-        <f>$B$2+9</f>
+        <f>$B$2+8</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 2편, 관련 동영상 링크 → 롱폼 #1</t>
+          <t>롱폼 #1 공개 (새 제목 공식, 썸네일 A/B 3종)</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>쇼츠→롱폼 클릭</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
@@ -1038,27 +1038,27 @@
         </is>
       </c>
       <c r="C15" s="8">
-        <f>$B$2+10</f>
+        <f>$B$2+9</f>
         <v/>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>팁 카드 1건 + 댓글 전체 답변</t>
+          <t>쇼츠 2편, 관련 동영상 링크 → 롱폼 #1</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>답변율 100%</t>
+          <t>쇼츠→롱폼 클릭</t>
         </is>
       </c>
       <c r="H15" s="9" t="n"/>
@@ -1077,27 +1077,27 @@
         </is>
       </c>
       <c r="C16" s="8">
-        <f>$B$2+11</f>
+        <f>$B$2+10</f>
         <v/>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #2 공개 (다른 시리즈, 썸네일 A/B)</t>
+          <t>팁 카드 1건 + 댓글 전체 답변</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>CTR 48h</t>
+          <t>답변율 100%</t>
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
@@ -1116,27 +1116,27 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>$B$2+12</f>
+        <f>$B$2+11</f>
         <v/>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>금</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 3편 (롱폼 #2 클립 + 훅형)</t>
+          <t>롱폼 #2 공개 (다른 시리즈, 썸네일 A/B)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 조회수</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H17" s="9" t="n"/>
@@ -1155,27 +1155,27 @@
         </is>
       </c>
       <c r="C18" s="8">
-        <f>$B$2+13</f>
+        <f>$B$2+12</f>
         <v/>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>주간 지표 기록, 저CTR 썸네일 교체</t>
+          <t>쇼츠 3편 (롱폼 #2 클립 + 훅형)</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W2</t>
+          <t>쇼츠 조회수</t>
         </is>
       </c>
       <c r="H18" s="9" t="n"/>
@@ -1185,36 +1185,36 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>글로벌·첫 7일 루틴</t>
+          <t>신규 콘텐츠 + A/B</t>
         </is>
       </c>
       <c r="C19" s="8">
-        <f>$B$2+14</f>
+        <f>$B$2+12</f>
         <v/>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>글로벌</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>상위 10개 영상 영어·일본어 제목·설명 입력</t>
+          <t>첫 앨범 10곡 제출, 팟캐스트 3편 등록, 스튜디오 RSS 연결</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>번역 메타 10편</t>
+          <t>발매 접수, 팟캐스트 탭</t>
         </is>
       </c>
       <c r="H19" s="9" t="n"/>
@@ -1224,36 +1224,36 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>글로벌·첫 7일 루틴</t>
+          <t>신규 콘텐츠 + A/B</t>
         </is>
       </c>
       <c r="C20" s="8">
-        <f>$B$2+15</f>
+        <f>$B$2+13</f>
         <v/>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #3 공개 + 첫 7일 체크리스트 D-0 실행</t>
+          <t>주간 지표 기록, 저CTR 썸네일 교체</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>체크리스트 완료</t>
+          <t>KPI 시트 W2</t>
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
@@ -1272,27 +1272,27 @@
         </is>
       </c>
       <c r="C21" s="8">
-        <f>$B$2+16</f>
+        <f>$B$2+14</f>
         <v/>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>배포</t>
+          <t>글로벌</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>인스타 릴스·맘카페·블로그 임베드</t>
+          <t>상위 10개 영상 영어·일본어 제목·설명 입력</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>외부 유입 수</t>
+          <t>번역 메타 10편</t>
         </is>
       </c>
       <c r="H21" s="9" t="n"/>
@@ -1311,27 +1311,27 @@
         </is>
       </c>
       <c r="C22" s="8">
-        <f>$B$2+17</f>
+        <f>$B$2+15</f>
         <v/>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Hype 요청 게시 (자격 충족 시) + 팁 카드</t>
+          <t>롱폼 #3 공개 + 첫 7일 체크리스트 D-0 실행</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>하이프 수</t>
+          <t>체크리스트 완료</t>
         </is>
       </c>
       <c r="H22" s="9" t="n"/>
@@ -1350,27 +1350,27 @@
         </is>
       </c>
       <c r="C23" s="8">
-        <f>$B$2+18</f>
+        <f>$B$2+16</f>
         <v/>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>배포</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #4 공개 (해외 타깃, KST 09:00 예약)</t>
+          <t>인스타 릴스·맘카페·블로그 임베드</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>해외 조회 비율</t>
+          <t>외부 유입 수</t>
         </is>
       </c>
       <c r="H23" s="9" t="n"/>
@@ -1389,27 +1389,27 @@
         </is>
       </c>
       <c r="C24" s="8">
-        <f>$B$2+19</f>
+        <f>$B$2+17</f>
         <v/>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 3편 (영어 자막 포함)</t>
+          <t>Hype 요청 게시 (자격 충족 시) + 팁 카드</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 조회수</t>
+          <t>하이프 수</t>
         </is>
       </c>
       <c r="H24" s="9" t="n"/>
@@ -1428,27 +1428,27 @@
         </is>
       </c>
       <c r="C25" s="8">
-        <f>$B$2+20</f>
+        <f>$B$2+18</f>
         <v/>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>금</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>초기 48시간 조회 추이 기록</t>
+          <t>롱폼 #4 공개 (해외 타깃, KST 09:00 예약)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W3</t>
+          <t>해외 조회 비율</t>
         </is>
       </c>
       <c r="H25" s="9" t="n"/>
@@ -1458,36 +1458,36 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>리뷰·재작성</t>
+          <t>글로벌·첫 7일 루틴</t>
         </is>
       </c>
       <c r="C26" s="8">
-        <f>$B$2+21</f>
+        <f>$B$2+19</f>
         <v/>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>분석</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>4주 지표 리뷰: 노출·CTR·AVD 전월 대비</t>
+          <t>쇼츠 3편 (영어 자막 포함)</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>리뷰 노트</t>
+          <t>쇼츠 조회수</t>
         </is>
       </c>
       <c r="H26" s="9" t="n"/>
@@ -1497,36 +1497,36 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>리뷰·재작성</t>
+          <t>글로벌·첫 7일 루틴</t>
         </is>
       </c>
       <c r="C27" s="8">
-        <f>$B$2+22</f>
+        <f>$B$2+19</f>
         <v/>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>분석</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>A/B 승자 썸네일 패턴 확정 → 가이드 반영</t>
+          <t>YouTube Music 반영 확인, OAC 신청, Spotify·Apple 등록</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>thumbnail_guide 갱신</t>
+          <t>Topic 채널 URL</t>
         </is>
       </c>
       <c r="H27" s="9" t="n"/>
@@ -1536,36 +1536,36 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>리뷰·재작성</t>
+          <t>글로벌·첫 7일 루틴</t>
         </is>
       </c>
       <c r="C28" s="8">
-        <f>$B$2+23</f>
+        <f>$B$2+20</f>
         <v/>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>재작성</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>저성과 영상 10편 제목·설명 재작성</t>
+          <t>초기 48시간 조회 추이 기록</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>check_metadata.py 통과</t>
+          <t>KPI 시트 W3</t>
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
@@ -1584,27 +1584,27 @@
         </is>
       </c>
       <c r="C29" s="8">
-        <f>$B$2+24</f>
+        <f>$B$2+21</f>
         <v/>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>분석</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #5 공개 (승자 패턴 적용)</t>
+          <t>4주 지표 리뷰: 노출·CTR·AVD 전월 대비</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>CTR 48h</t>
+          <t>리뷰 노트</t>
         </is>
       </c>
       <c r="H29" s="9" t="n"/>
@@ -1623,27 +1623,27 @@
         </is>
       </c>
       <c r="C30" s="8">
-        <f>$B$2+25</f>
+        <f>$B$2+22</f>
         <v/>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>분석</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>후기 공유 + 다음 달 라인업 설문</t>
+          <t>A/B 승자 썸네일 패턴 확정 → 가이드 반영</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>응답 수</t>
+          <t>thumbnail_guide 갱신</t>
         </is>
       </c>
       <c r="H30" s="9" t="n"/>
@@ -1662,27 +1662,27 @@
         </is>
       </c>
       <c r="C31" s="8">
-        <f>$B$2+26</f>
+        <f>$B$2+23</f>
         <v/>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>재작성</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 2편</t>
+          <t>저성과 영상 10편 제목·설명 재작성</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 조회수</t>
+          <t>check_metadata.py 통과</t>
         </is>
       </c>
       <c r="H31" s="9" t="n"/>
@@ -1701,27 +1701,27 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>$B$2+27</f>
+        <f>$B$2+24</f>
         <v/>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>월간 KPI 마감, 다음 4주 계획 초안</t>
+          <t>롱폼 #5 공개 (승자 패턴 적용)</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W4</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H32" s="9" t="n"/>
@@ -1729,73 +1729,229 @@
       <c r="J32" s="9" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-      <c r="J33" s="2" t="n"/>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>리뷰·재작성</t>
+        </is>
+      </c>
+      <c r="C33" s="8">
+        <f>$B$2+25</f>
+        <v/>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>금</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>커뮤니티</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>후기 공유 + 다음 달 라인업 설문</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>응답 수</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="9" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>리뷰·재작성</t>
+        </is>
+      </c>
+      <c r="C34" s="8">
+        <f>$B$2+26</f>
+        <v/>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>토</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>쇼츠</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>쇼츠 2편</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>쇼츠 조회수</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>리뷰·재작성</t>
+        </is>
+      </c>
+      <c r="C35" s="8">
+        <f>$B$2+26</f>
+        <v/>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>토</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>유통</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>트래픽 소스에 YouTube Music·팟캐스트 항목 생겼는지 확인</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>KPI 시트 W4</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>리뷰·재작성</t>
+        </is>
+      </c>
+      <c r="C36" s="8">
+        <f>$B$2+27</f>
+        <v/>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>측정</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>월간 KPI 마감, 다음 4주 계획 초안</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>KPI 시트 W4</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>완료 건수</t>
         </is>
       </c>
-      <c r="B34" s="2">
-        <f>COUNTIF(I5:I32,"Y")</f>
-        <v/>
-      </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="B38" s="2">
+        <f>COUNTIF(I5:I36,"Y")</f>
+        <v/>
+      </c>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>전체 건수</t>
         </is>
       </c>
-      <c r="B35" s="2">
-        <f>COUNTA(F5:F32)</f>
-        <v/>
-      </c>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="B39" s="2">
+        <f>COUNTA(F5:F36)</f>
+        <v/>
+      </c>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>진행률</t>
         </is>
       </c>
-      <c r="B36" s="10">
-        <f>IF(B35=0,0,B34/B35)</f>
-        <v/>
-      </c>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
+      <c r="B40" s="10">
+        <f>IF(B39=0,0,B38/B39)</f>
+        <v/>
+      </c>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1864,15 +2020,15 @@
         </is>
       </c>
       <c r="C2" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A2,'4주 캘린더'!$E$5:$E$32,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A2,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
         <v/>
       </c>
       <c r="D2" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A2,'4주 캘린더'!$E$5:$E$32,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A2,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
         <v/>
       </c>
       <c r="E2" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A2,'4주 캘린더'!$E$5:$E$32,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A2,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F2" s="11" t="inlineStr">
@@ -1893,15 +2049,15 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A3,'4주 캘린더'!$E$5:$E$32,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A3,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A3,'4주 캘린더'!$E$5:$E$32,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A3,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
         <v/>
       </c>
       <c r="E3" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A3,'4주 캘린더'!$E$5:$E$32,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A3,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F3" s="11" t="inlineStr">
@@ -1922,15 +2078,15 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A4,'4주 캘린더'!$E$5:$E$32,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A4,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A4,'4주 캘린더'!$E$5:$E$32,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A4,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A4,'4주 캘린더'!$E$5:$E$32,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A4,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F4" s="11" t="inlineStr">
@@ -1951,15 +2107,15 @@
         </is>
       </c>
       <c r="C5" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A5,'4주 캘린더'!$E$5:$E$32,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A5,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A5,'4주 캘린더'!$E$5:$E$32,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A5,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$32,A5,'4주 캘린더'!$E$5:$E$32,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A5,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F5" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Add channel split plan: sleep music moves to a new channel
- plans/channel_split_plan_20260917.md: constraints, new-channel setup
  table, content migration (6 long-forms re-uploaded in measured order,
  10h new build, 33 two-minute tracks become the distribution album, 39
  videos unlisted on @PPAIEO), 8-week schedule, first-28-day targets
- Plan v2 and analysis report record the decision; calendar W1 replaced
  with setup and migration tasks (33 rows, formulas verified)
- README rows for analysis and split plan

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C2dffSHYa7wwyhksGy8dMJ
</commit_message>
<xml_diff>
--- a/calendar/4week_calendar.xlsx
+++ b/calendar/4week_calendar.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -632,7 +632,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C5" s="8">
@@ -646,17 +646,17 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>점검</t>
+          <t>개설</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>전 영상 시청자층(아동용 여부) 전수 확인</t>
+          <t>브랜드 계정으로 새 채널 개설, 채널명·핸들·설명·키워드·시청자층(아동용 아님)·업로드 기본값 설정</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>체크 결과 시트</t>
+          <t>channel_split_plan 1장 체크</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
@@ -683,31 +683,31 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C6" s="8">
-        <f>$B$2+1</f>
+        <f>$B$2+0</f>
         <v/>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>점검</t>
+          <t>정리</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>재생목록 5개 구성, 전 영상 배치</t>
+          <t>@PPAIEO 수면음악 39편 일부공개 전환, 재생목록 삭제, 채널 키워드 정리</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>재생목록 링크</t>
+          <t>일부공개 39편</t>
         </is>
       </c>
       <c r="H6" s="9" t="n"/>
@@ -722,31 +722,31 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C7" s="8">
-        <f>$B$2+2</f>
+        <f>$B$2+1</f>
         <v/>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>점검</t>
+          <t>세팅</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>최종화면·타임스탬프 미설정 영상 보완</t>
+          <t>새 채널 재생목록 5개 생성, 배너·프로필 업로드</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>check_metadata.py 통과</t>
+          <t>재생목록 링크</t>
         </is>
       </c>
       <c r="H7" s="9" t="n"/>
@@ -761,31 +761,31 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C8" s="8">
-        <f>$B$2+3</f>
+        <f>$B$2+1</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>제작</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>썸네일 가이드 확정, 기존 상위 5개 썸네일 재제작</t>
+          <t>롱폼 1번(엄마 허밍 3시간) 재작업 후 예약 공개 20:00, 썸네일 A/B 3종</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>썸네일 3종×5</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H8" s="9" t="n"/>
@@ -800,31 +800,31 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C9" s="8">
-        <f>$B$2+4</f>
+        <f>$B$2+2</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>세팅</t>
+          <t>제작</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>24시간 라이브 스트림 세팅·테스트</t>
+          <t>롱폼 2번(무가사 3시간) 제목·썸네일·다국어 메타 재작업</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>라이브 URL</t>
+          <t>check_metadata.py 통과</t>
         </is>
       </c>
       <c r="H9" s="9" t="n"/>
@@ -839,31 +839,31 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C10" s="8">
-        <f>$B$2+5</f>
+        <f>$B$2+3</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>제작</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>설문: 이번 주 소리 투표</t>
+          <t>30분 무가사 첫 10분 재편집(오디오 사양 2장)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>응답 수</t>
+          <t>재편집 파일</t>
         </is>
       </c>
       <c r="H10" s="9" t="n"/>
@@ -878,31 +878,31 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C11" s="8">
-        <f>$B$2+5</f>
+        <f>$B$2+4</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>금</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>유통</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>음원 출처 정리(자체 제작·독점만), 유통사·팟캐스트 호스팅 계정 개설</t>
+          <t>롱폼 2번 예약 공개 20:00, 최종화면 1번↔2번 상호 연결</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>출처표, 계정</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H11" s="9" t="n"/>
@@ -917,31 +917,31 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C12" s="8">
-        <f>$B$2+6</f>
+        <f>$B$2+5</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>기준선 기록: 노출·CTR·AVD·트래픽 소스</t>
+          <t>2분짜리 33곡을 허밍·무가사 앨범 2장으로 정리, 유통사·팟캐스트 호스팅 계정 개설</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W0</t>
+          <t>트랙 목록, 계정</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
@@ -951,36 +951,36 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>신규 콘텐츠 + A/B</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C13" s="8">
-        <f>$B$2+7</f>
+        <f>$B$2+6</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>설문 결과 발표 + 화요일 공개 예고</t>
+          <t>새 채널 첫 주 지표·@PPAIEO 트래픽 소스 기준선 기록</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>게시글</t>
+          <t>KPI 시트 W0</t>
         </is>
       </c>
       <c r="H13" s="9" t="n"/>
@@ -999,27 +999,27 @@
         </is>
       </c>
       <c r="C14" s="8">
-        <f>$B$2+8</f>
+        <f>$B$2+7</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #1 공개 (새 제목 공식, 썸네일 A/B 3종)</t>
+          <t>설문 결과 발표 + 화요일 공개 예고</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>CTR 48h</t>
+          <t>게시글</t>
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
@@ -1038,27 +1038,27 @@
         </is>
       </c>
       <c r="C15" s="8">
-        <f>$B$2+9</f>
+        <f>$B$2+8</f>
         <v/>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 2편, 관련 동영상 링크 → 롱폼 #1</t>
+          <t>롱폼 #1 공개 (새 제목 공식, 썸네일 A/B 3종)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>쇼츠→롱폼 클릭</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H15" s="9" t="n"/>
@@ -1077,27 +1077,27 @@
         </is>
       </c>
       <c r="C16" s="8">
-        <f>$B$2+10</f>
+        <f>$B$2+9</f>
         <v/>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>팁 카드 1건 + 댓글 전체 답변</t>
+          <t>쇼츠 2편, 관련 동영상 링크 → 롱폼 #1</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>답변율 100%</t>
+          <t>쇼츠→롱폼 클릭</t>
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
@@ -1116,27 +1116,27 @@
         </is>
       </c>
       <c r="C17" s="8">
-        <f>$B$2+11</f>
+        <f>$B$2+10</f>
         <v/>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #2 공개 (다른 시리즈, 썸네일 A/B)</t>
+          <t>팁 카드 1건 + 댓글 전체 답변</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>CTR 48h</t>
+          <t>답변율 100%</t>
         </is>
       </c>
       <c r="H17" s="9" t="n"/>
@@ -1155,27 +1155,27 @@
         </is>
       </c>
       <c r="C18" s="8">
-        <f>$B$2+12</f>
+        <f>$B$2+11</f>
         <v/>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>금</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 3편 (롱폼 #2 클립 + 훅형)</t>
+          <t>롱폼 #2 공개 (다른 시리즈, 썸네일 A/B)</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 조회수</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H18" s="9" t="n"/>
@@ -1204,17 +1204,17 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>유통</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>첫 앨범 10곡 제출, 팟캐스트 3편 등록, 스튜디오 RSS 연결</t>
+          <t>쇼츠 3편 (롱폼 #2 클립 + 훅형)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>발매 접수, 팟캐스트 탭</t>
+          <t>쇼츠 조회수</t>
         </is>
       </c>
       <c r="H19" s="9" t="n"/>
@@ -1233,27 +1233,27 @@
         </is>
       </c>
       <c r="C20" s="8">
-        <f>$B$2+13</f>
+        <f>$B$2+12</f>
         <v/>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>주간 지표 기록, 저CTR 썸네일 교체</t>
+          <t>첫 앨범 10곡 제출, 팟캐스트 3편 등록, 스튜디오 RSS 연결</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W2</t>
+          <t>발매 접수, 팟캐스트 탭</t>
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
@@ -1263,36 +1263,36 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>글로벌·첫 7일 루틴</t>
+          <t>신규 콘텐츠 + A/B</t>
         </is>
       </c>
       <c r="C21" s="8">
-        <f>$B$2+14</f>
+        <f>$B$2+13</f>
         <v/>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>글로벌</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>상위 10개 영상 영어·일본어 제목·설명 입력</t>
+          <t>주간 지표 기록, 저CTR 썸네일 교체</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>번역 메타 10편</t>
+          <t>KPI 시트 W2</t>
         </is>
       </c>
       <c r="H21" s="9" t="n"/>
@@ -1311,27 +1311,27 @@
         </is>
       </c>
       <c r="C22" s="8">
-        <f>$B$2+15</f>
+        <f>$B$2+14</f>
         <v/>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>글로벌</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #3 공개 + 첫 7일 체크리스트 D-0 실행</t>
+          <t>상위 10개 영상 영어·일본어 제목·설명 입력</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>체크리스트 완료</t>
+          <t>번역 메타 10편</t>
         </is>
       </c>
       <c r="H22" s="9" t="n"/>
@@ -1350,27 +1350,27 @@
         </is>
       </c>
       <c r="C23" s="8">
-        <f>$B$2+16</f>
+        <f>$B$2+15</f>
         <v/>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>배포</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>인스타 릴스·맘카페·블로그 임베드</t>
+          <t>롱폼 #3 공개 + 첫 7일 체크리스트 D-0 실행</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>외부 유입 수</t>
+          <t>체크리스트 완료</t>
         </is>
       </c>
       <c r="H23" s="9" t="n"/>
@@ -1389,27 +1389,27 @@
         </is>
       </c>
       <c r="C24" s="8">
-        <f>$B$2+17</f>
+        <f>$B$2+16</f>
         <v/>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>배포</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Hype 요청 게시 (자격 충족 시) + 팁 카드</t>
+          <t>인스타 릴스·맘카페·블로그 임베드</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>하이프 수</t>
+          <t>외부 유입 수</t>
         </is>
       </c>
       <c r="H24" s="9" t="n"/>
@@ -1428,27 +1428,27 @@
         </is>
       </c>
       <c r="C25" s="8">
-        <f>$B$2+18</f>
+        <f>$B$2+17</f>
         <v/>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #4 공개 (해외 타깃, KST 09:00 예약)</t>
+          <t>Hype 요청 게시 (자격 충족 시) + 팁 카드</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>해외 조회 비율</t>
+          <t>하이프 수</t>
         </is>
       </c>
       <c r="H25" s="9" t="n"/>
@@ -1467,27 +1467,27 @@
         </is>
       </c>
       <c r="C26" s="8">
-        <f>$B$2+19</f>
+        <f>$B$2+18</f>
         <v/>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>금</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 3편 (영어 자막 포함)</t>
+          <t>롱폼 #4 공개 (해외 타깃, KST 09:00 예약)</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 조회수</t>
+          <t>해외 조회 비율</t>
         </is>
       </c>
       <c r="H26" s="9" t="n"/>
@@ -1516,17 +1516,17 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>유통</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>YouTube Music 반영 확인, OAC 신청, Spotify·Apple 등록</t>
+          <t>쇼츠 3편 (영어 자막 포함)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Topic 채널 URL</t>
+          <t>쇼츠 조회수</t>
         </is>
       </c>
       <c r="H27" s="9" t="n"/>
@@ -1545,27 +1545,27 @@
         </is>
       </c>
       <c r="C28" s="8">
-        <f>$B$2+20</f>
+        <f>$B$2+19</f>
         <v/>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>초기 48시간 조회 추이 기록</t>
+          <t>YouTube Music 반영 확인, OAC 신청, Spotify·Apple 등록</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W3</t>
+          <t>Topic 채널 URL</t>
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
@@ -1575,36 +1575,36 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>리뷰·재작성</t>
+          <t>글로벌·첫 7일 루틴</t>
         </is>
       </c>
       <c r="C29" s="8">
-        <f>$B$2+21</f>
+        <f>$B$2+20</f>
         <v/>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>월</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>분석</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>4주 지표 리뷰: 노출·CTR·AVD 전월 대비</t>
+          <t>초기 48시간 조회 추이 기록</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>리뷰 노트</t>
+          <t>KPI 시트 W3</t>
         </is>
       </c>
       <c r="H29" s="9" t="n"/>
@@ -1623,12 +1623,12 @@
         </is>
       </c>
       <c r="C30" s="8">
-        <f>$B$2+22</f>
+        <f>$B$2+21</f>
         <v/>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>화</t>
+          <t>월</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>A/B 승자 썸네일 패턴 확정 → 가이드 반영</t>
+          <t>4주 지표 리뷰: 노출·CTR·AVD 전월 대비</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>thumbnail_guide 갱신</t>
+          <t>리뷰 노트</t>
         </is>
       </c>
       <c r="H30" s="9" t="n"/>
@@ -1662,27 +1662,27 @@
         </is>
       </c>
       <c r="C31" s="8">
-        <f>$B$2+23</f>
+        <f>$B$2+22</f>
         <v/>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>수</t>
+          <t>화</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>재작성</t>
+          <t>분석</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>저성과 영상 10편 제목·설명 재작성</t>
+          <t>A/B 승자 썸네일 패턴 확정 → 가이드 반영</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>check_metadata.py 통과</t>
+          <t>thumbnail_guide 갱신</t>
         </is>
       </c>
       <c r="H31" s="9" t="n"/>
@@ -1701,27 +1701,27 @@
         </is>
       </c>
       <c r="C32" s="8">
-        <f>$B$2+24</f>
+        <f>$B$2+23</f>
         <v/>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>목</t>
+          <t>수</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>업로드</t>
+          <t>재작성</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>롱폼 #5 공개 (승자 패턴 적용)</t>
+          <t>저성과 영상 10편 제목·설명 재작성</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>CTR 48h</t>
+          <t>check_metadata.py 통과</t>
         </is>
       </c>
       <c r="H32" s="9" t="n"/>
@@ -1740,27 +1740,27 @@
         </is>
       </c>
       <c r="C33" s="8">
-        <f>$B$2+25</f>
+        <f>$B$2+24</f>
         <v/>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>금</t>
+          <t>목</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>커뮤니티</t>
+          <t>업로드</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>후기 공유 + 다음 달 라인업 설문</t>
+          <t>롱폼 #5 공개 (승자 패턴 적용)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>응답 수</t>
+          <t>CTR 48h</t>
         </is>
       </c>
       <c r="H33" s="9" t="n"/>
@@ -1779,27 +1779,27 @@
         </is>
       </c>
       <c r="C34" s="8">
-        <f>$B$2+26</f>
+        <f>$B$2+25</f>
         <v/>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>토</t>
+          <t>금</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>쇼츠</t>
+          <t>커뮤니티</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 2편</t>
+          <t>후기 공유 + 다음 달 라인업 설문</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>쇼츠 조회수</t>
+          <t>응답 수</t>
         </is>
       </c>
       <c r="H34" s="9" t="n"/>
@@ -1828,17 +1828,17 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>유통</t>
+          <t>쇼츠</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>트래픽 소스에 YouTube Music·팟캐스트 항목 생겼는지 확인</t>
+          <t>쇼츠 2편</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>KPI 시트 W4</t>
+          <t>쇼츠 조회수</t>
         </is>
       </c>
       <c r="H35" s="9" t="n"/>
@@ -1857,22 +1857,22 @@
         </is>
       </c>
       <c r="C36" s="8">
-        <f>$B$2+27</f>
+        <f>$B$2+26</f>
         <v/>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>토</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>유통</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>월간 KPI 마감, 다음 4주 계획 초안</t>
+          <t>트래픽 소스에 YouTube Music·팟캐스트 항목 생겼는지 확인</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -1885,27 +1885,47 @@
       <c r="J36" s="9" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>리뷰·재작성</t>
+        </is>
+      </c>
+      <c r="C37" s="8">
+        <f>$B$2+27</f>
+        <v/>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>측정</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>월간 KPI 마감, 다음 4주 계획 초안</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>KPI 시트 W4</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>완료 건수</t>
-        </is>
-      </c>
-      <c r="B38" s="2">
-        <f>COUNTIF(I5:I36,"Y")</f>
-        <v/>
-      </c>
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="n"/>
       <c r="D38" s="2" t="n"/>
       <c r="E38" s="2" t="n"/>
@@ -1918,11 +1938,11 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>전체 건수</t>
+          <t>완료 건수</t>
         </is>
       </c>
       <c r="B39" s="2">
-        <f>COUNTA(F5:F36)</f>
+        <f>COUNTIF(I5:I37,"Y")</f>
         <v/>
       </c>
       <c r="C39" s="2" t="n"/>
@@ -1937,11 +1957,11 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>진행률</t>
-        </is>
-      </c>
-      <c r="B40" s="10">
-        <f>IF(B39=0,0,B38/B39)</f>
+          <t>전체 건수</t>
+        </is>
+      </c>
+      <c r="B40" s="2">
+        <f>COUNTA(F5:F37)</f>
         <v/>
       </c>
       <c r="C40" s="2" t="n"/>
@@ -1952,6 +1972,25 @@
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="2" t="n"/>
       <c r="J40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>진행률</t>
+        </is>
+      </c>
+      <c r="B41" s="10">
+        <f>IF(B40=0,0,B39/B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2016,19 +2055,19 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>점검·세팅</t>
+          <t>채널 개설·이관</t>
         </is>
       </c>
       <c r="C2" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A2,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A2,'4주 캘린더'!$E$5:$E$37,"업로드")</f>
         <v/>
       </c>
       <c r="D2" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A2,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A2,'4주 캘린더'!$E$5:$E$37,"쇼츠")</f>
         <v/>
       </c>
       <c r="E2" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A2,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A2,'4주 캘린더'!$E$5:$E$37,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F2" s="11" t="inlineStr">
@@ -2049,15 +2088,15 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A3,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A3,'4주 캘린더'!$E$5:$E$37,"업로드")</f>
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A3,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A3,'4주 캘린더'!$E$5:$E$37,"쇼츠")</f>
         <v/>
       </c>
       <c r="E3" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A3,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A3,'4주 캘린더'!$E$5:$E$37,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F3" s="11" t="inlineStr">
@@ -2078,15 +2117,15 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A4,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A4,'4주 캘린더'!$E$5:$E$37,"업로드")</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A4,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A4,'4주 캘린더'!$E$5:$E$37,"쇼츠")</f>
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A4,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A4,'4주 캘린더'!$E$5:$E$37,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F4" s="11" t="inlineStr">
@@ -2107,15 +2146,15 @@
         </is>
       </c>
       <c r="C5" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A5,'4주 캘린더'!$E$5:$E$36,"업로드")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A5,'4주 캘린더'!$E$5:$E$37,"업로드")</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A5,'4주 캘린더'!$E$5:$E$36,"쇼츠")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A5,'4주 캘린더'!$E$5:$E$37,"쇼츠")</f>
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>COUNTIFS('4주 캘린더'!$A$5:$A$36,A5,'4주 캘린더'!$E$5:$E$36,"커뮤니티")</f>
+        <f>COUNTIFS('4주 캘린더'!$A$5:$A$37,A5,'4주 캘린더'!$E$5:$E$37,"커뮤니티")</f>
         <v/>
       </c>
       <c r="F5" s="11" t="inlineStr">

</xml_diff>